<commit_message>
Got all data uploaded to database
</commit_message>
<xml_diff>
--- a/database/specimens_long_filtered.xlsx
+++ b/database/specimens_long_filtered.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hensley/Desktop/wiscam_database/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFFFC5BB-E6A6-834F-A4EF-6E061CF7D07A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6BAF92-069E-C04E-B695-5492AEE1641A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33460" yWindow="2320" windowWidth="29400" windowHeight="18440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="-2480" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="specimens" sheetId="1" r:id="rId1"/>
@@ -23,12 +23,25 @@
     <sheet name="universal_veil_stipe_base" sheetId="8" r:id="rId8"/>
     <sheet name="basal_bulb" sheetId="9" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5655" uniqueCount="654">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5655" uniqueCount="656">
   <si>
     <t>specimenid</t>
   </si>
@@ -1968,12 +1981,15 @@
     <t>eastern hemlock (Tsuga canadensis)</t>
   </si>
   <si>
+    <t>white pine (Pinus strobus)</t>
+  </si>
+  <si>
+    <t>red pine (Pinus resinosa)</t>
+  </si>
+  <si>
     <t>white pine (pine (Pinus) strobus)</t>
   </si>
   <si>
-    <t>red pine (pine (Pinus) resinosa)</t>
-  </si>
-  <si>
     <t>pine (Pinus)</t>
   </si>
   <si>
@@ -1990,6 +2006,9 @@
   </si>
   <si>
     <t>large toothed aspen (Populus deltoides)</t>
+  </si>
+  <si>
+    <t>Franklin nature trail</t>
   </si>
 </sst>
 </file>
@@ -2508,7 +2527,7 @@
         <v>643</v>
       </c>
       <c r="F5" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="G5" t="s">
         <v>35</v>
@@ -2773,7 +2792,7 @@
         <v>645</v>
       </c>
       <c r="F13" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="G13" t="s">
         <v>68</v>
@@ -2843,7 +2862,7 @@
         <v>645</v>
       </c>
       <c r="F15" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="G15" t="s">
         <v>77</v>
@@ -2875,7 +2894,7 @@
         <v>15</v>
       </c>
       <c r="E16" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="F16" t="s">
         <v>645</v>
@@ -2910,10 +2929,10 @@
         <v>15</v>
       </c>
       <c r="E17" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="F17" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="G17" t="s">
         <v>86</v>
@@ -2945,7 +2964,7 @@
         <v>15</v>
       </c>
       <c r="E18" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="F18" t="s">
         <v>645</v>
@@ -2980,10 +2999,10 @@
         <v>15</v>
       </c>
       <c r="E19" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="F19" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="G19" t="s">
         <v>94</v>
@@ -3015,7 +3034,7 @@
         <v>97</v>
       </c>
       <c r="E20" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="G20" t="s">
         <v>98</v>
@@ -3047,7 +3066,7 @@
         <v>15</v>
       </c>
       <c r="E21" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="G21" t="s">
         <v>103</v>
@@ -3079,10 +3098,10 @@
         <v>15</v>
       </c>
       <c r="E22" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="F22" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="G22" t="s">
         <v>109</v>
@@ -3114,7 +3133,7 @@
         <v>15</v>
       </c>
       <c r="E23" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="G23" t="s">
         <v>113</v>
@@ -3158,7 +3177,7 @@
         <v>122</v>
       </c>
       <c r="J24" t="s">
-        <v>123</v>
+        <v>655</v>
       </c>
       <c r="K24" t="s">
         <v>124</v>
@@ -3274,7 +3293,7 @@
         <v>15</v>
       </c>
       <c r="E28" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="F28" t="s">
         <v>639</v>
@@ -3309,7 +3328,7 @@
         <v>15</v>
       </c>
       <c r="E29" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="F29" t="s">
         <v>639</v>
@@ -3344,7 +3363,7 @@
         <v>15</v>
       </c>
       <c r="E30" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="F30" t="s">
         <v>639</v>
@@ -3379,7 +3398,7 @@
         <v>15</v>
       </c>
       <c r="E31" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="F31" t="s">
         <v>639</v>
@@ -3414,7 +3433,7 @@
         <v>15</v>
       </c>
       <c r="E32" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="F32" t="s">
         <v>639</v>
@@ -3449,7 +3468,7 @@
         <v>15</v>
       </c>
       <c r="E33" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="F33" t="s">
         <v>639</v>
@@ -3484,7 +3503,7 @@
         <v>15</v>
       </c>
       <c r="E34" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="F34" t="s">
         <v>639</v>
@@ -3519,7 +3538,7 @@
         <v>15</v>
       </c>
       <c r="E35" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="F35" t="s">
         <v>639</v>
@@ -3813,7 +3832,7 @@
         <v>645</v>
       </c>
       <c r="F44" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="G44" t="s">
         <v>180</v>
@@ -3848,7 +3867,7 @@
         <v>645</v>
       </c>
       <c r="F45" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="G45" t="s">
         <v>180</v>
@@ -4110,7 +4129,7 @@
         <v>15</v>
       </c>
       <c r="E53" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="F53" t="s">
         <v>645</v>
@@ -4145,7 +4164,7 @@
         <v>15</v>
       </c>
       <c r="E54" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="F54" t="s">
         <v>645</v>
@@ -4279,7 +4298,7 @@
         <v>15</v>
       </c>
       <c r="E58" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="G58" t="s">
         <v>240</v>
@@ -4311,7 +4330,7 @@
         <v>15</v>
       </c>
       <c r="E59" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="G59" t="s">
         <v>244</v>
@@ -4343,7 +4362,7 @@
         <v>15</v>
       </c>
       <c r="E60" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="G60" t="s">
         <v>247</v>
@@ -4375,7 +4394,7 @@
         <v>15</v>
       </c>
       <c r="E61" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="G61" t="s">
         <v>250</v>
@@ -4407,7 +4426,7 @@
         <v>15</v>
       </c>
       <c r="E62" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="G62" t="s">
         <v>253</v>
@@ -4439,7 +4458,7 @@
         <v>15</v>
       </c>
       <c r="E63" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="G63" t="s">
         <v>256</v>
@@ -4471,7 +4490,7 @@
         <v>15</v>
       </c>
       <c r="E64" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="G64" t="s">
         <v>256</v>
@@ -4675,7 +4694,7 @@
         <v>645</v>
       </c>
       <c r="F70" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="G70" t="s">
         <v>281</v>

</xml_diff>